<commit_message>
docs(release): sync 0.5.3 verification evidence
</commit_message>
<xml_diff>
--- a/docs/user-story-status.xlsx
+++ b/docs/user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R90804bf896a94aa6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="User Stories" sheetId="2" r:id="R5959f7dd51a347bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Log" sheetId="3" r:id="R034db2b31ddd4432"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Errors" sheetId="4" r:id="R83c7010a12ce4d87"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Re2d0b41121ac4f6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="User Stories" sheetId="2" r:id="R0a91f89bb4164355"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Log" sheetId="3" r:id="R6f63744b893545df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Errors" sheetId="4" r:id="R37cd54e3463d41c9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -428,7 +428,7 @@
         <x:v>Generated</x:v>
       </x:c>
       <x:c r="B3" s="4" t="str">
-        <x:v>2026-07-13</x:v>
+        <x:v>2026-07-14</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -475,10 +475,9 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="3" t="str">
-        <x:v>Not run</x:v>
+        <x:v>User-waived</x:v>
       </x:c>
       <x:c r="B9" s="4" t="n">
-        <x:f>COUNTIF('User Stories'!G4:G200,"NOT RUN")</x:f>
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -1296,11 +1295,11 @@
         <x:v>PARTIAL</x:v>
       </x:c>
       <x:c r="H27" s="4" t="str">
-        <x:v>All 12,994 exact keys plus 71 normalized-source conflicts matched baseline semantics; scoped real Cavalry smoke proved the three top-level menus, but did not traverse every dialog/status surface.</x:v>
+        <x:v>All 12,994 exact keys plus 71 normalized-source conflicts matched baseline semantics. Scoped real Cavalry smoke proved the three top-level menus; zh-Hans, zh-Hant, and ja_JP empty-state hints were visually verified as translated, visible, horizontally centered, and free of trailing CJK full stops. The wider matrix was explicitly user-waived.</x:v>
       </x:c>
       <x:c r="I27" s="4"/>
       <x:c r="J27" s="15" t="str">
-        <x:v>Partially verified; full matrix not run</x:v>
+        <x:v>Partially verified; wider matrix user-waived</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -1320,19 +1319,19 @@
         <x:v>docs/workflows/cavalry-full-ui-100; tools/run_live_full_ui_matrix.js; tools/check_full_ui_matrix.js</x:v>
       </x:c>
       <x:c r="F28" s="4" t="str">
-        <x:v>Session-scoped live Cavalry.app 100% gate (not run)</x:v>
+        <x:v>Session-scoped live Cavalry.app 100% gate (user-waived 2026-07-14)</x:v>
       </x:c>
       <x:c r="G28" s="4" t="str">
-        <x:v>NOT RUN</x:v>
+        <x:v>USER-WAIVED</x:v>
       </x:c>
       <x:c r="H28" s="4" t="str">
-        <x:v>The session-scoped 100% full UI matrix was not run. The real three-language injector smoke is narrower evidence and is not relabeled as full coverage.</x:v>
+        <x:v>The maintainer explicitly waived the extra session-scoped 100% full UI matrix on 2026-07-14 after the real three-language injector smoke and targeted empty-state verification. Narrower evidence remains labeled as narrower evidence and is not relabeled as full coverage.</x:v>
       </x:c>
       <x:c r="I28" s="4" t="str">
         <x:v>E-004</x:v>
       </x:c>
       <x:c r="J28" s="15" t="str">
-        <x:v>Release gate not run</x:v>
+        <x:v>Maintainer waiver recorded; no 100% coverage claim</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -1492,7 +1491,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R563bd376bc9446ca"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c90869f2d784130"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1621,7 +1620,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="E7" s="4" t="str">
-        <x:v>Built Cavalry Language Switcher.app and Cavalry Language Switcher_0.5.2_aarch64.dmg from the final injector artifact.</x:v>
+        <x:v>Built Cavalry Language Switcher.app and Cavalry Language Switcher_0.5.3_aarch64.dmg from the final injector artifact.</x:v>
       </x:c>
       <x:c r="F7" s="15" t="str">
         <x:v>Notarization warning is expected for this explicitly ad-hoc signed release.</x:v>
@@ -1715,16 +1714,16 @@
         <x:v>US-25</x:v>
       </x:c>
       <x:c r="C12" s="4" t="str">
-        <x:v>node tools/run_live_full_ui_matrix.js --help</x:v>
+        <x:v>Extra session-scoped full UI matrix</x:v>
       </x:c>
       <x:c r="D12" s="4" t="str">
-        <x:v>PASS</x:v>
+        <x:v>USER-WAIVED</x:v>
       </x:c>
       <x:c r="E12" s="4" t="str">
-        <x:v>Help exits without starting Cavalry.</x:v>
+        <x:v>The maintainer explicitly waived the extra matrix on 2026-07-14; the incomplete clone/session run was terminated and deleted. Targeted zh-Hans, zh-Hant, and ja_JP empty-state visual checks passed.</x:v>
       </x:c>
       <x:c r="F12" s="15" t="str">
-        <x:v>The full UI matrix itself remains NOT RUN.</x:v>
+        <x:v>Real injection smoke and targeted empty-state evidence remain narrower and are not presented as 100% coverage; all three empty-state strings are centered and omit the trailing CJK full stop.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -1761,7 +1760,7 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="E14" s="4" t="str">
-        <x:v>Real-clone apply times: zh-Hans 2.512s, repeat 1.875s, zh-Hant 2.023s, ja_JP 2.268s; real Cavalry then passed all three menu sentinels per language.</x:v>
+        <x:v>Final 0.5.3 real-clone apply times: zh-Hans 1.824s, repeat 1.593s, zh-Hant 1.603s, ja_JP 1.788s; real Cavalry then passed all three menu sentinels per target language.</x:v>
       </x:c>
       <x:c r="F14" s="4" t="str">
         <x:v>PID/session/bundle hash plus inventory/log SHA-256 were recorded; /Applications critical bytes stayed identical and no process remained.</x:v>
@@ -1801,16 +1800,16 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="E16" s="4" t="str">
-        <x:v>Universal arm64+x86_64 dylib, SHA-256 eef1ca71daec699888530a755dea6c3fb89b508612a9910f65b5ba0aa16360eb, ad-hoc signed.</x:v>
+        <x:v>Universal arm64+x86_64 dylib, 2,337,536 bytes, SHA-256 2de7206c019da67a3ed831b44ca10498791a0bdab96bda23d8f8aecadba0c029, ad-hoc signed.</x:v>
       </x:c>
       <x:c r="F16" s="4" t="str">
-        <x:v>Both slices use @loader_path plus target Frameworks and contain no qt_sdk runtime RPATH.</x:v>
+        <x:v>Both slices use @loader_path plus target Frameworks and contain no qt_sdk runtime RPATH; packaged resource hash matches.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4521f5628ce24b3b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R54e268bab5224d88"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1984,19 +1983,19 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="E7" s="4" t="str">
-        <x:v>Not Run</x:v>
+        <x:v>User Waived</x:v>
       </x:c>
       <x:c r="F7" s="4" t="str">
-        <x:v>The full session-scoped 100% live UI matrix was not executed.</x:v>
+        <x:v>The extra session-scoped 100% live UI matrix was not completed before release.</x:v>
       </x:c>
       <x:c r="G7" s="4" t="str">
-        <x:v>This performance task proves injector semantics, real top-level menus, and runtime provenance, but does not navigate every live dialog and status surface.</x:v>
+        <x:v>The maintainer explicitly waived this wider matrix on 2026-07-14 after real three-language injection and targeted empty-state verification.</x:v>
       </x:c>
       <x:c r="H7" s="4" t="str">
-        <x:v>Keep the full matrix as an explicit release gate; never rename narrower smoke evidence as 100% coverage.</x:v>
+        <x:v>Record the waiver explicitly and never rename narrower smoke evidence as 100% coverage.</x:v>
       </x:c>
       <x:c r="I7" s="15" t="str">
-        <x:v>Real three-language injection passed; full matrix remains honestly NOT RUN.</x:v>
+        <x:v>Real three-language injection and targeted empty-state checks passed; wider matrix is USER-WAIVED.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -2089,7 +2088,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83b9293859a0406a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R370ef3a006ae449a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>